<commit_message>
風速計On/Offをハードスイッチ(PD3/TPS22965)で制御 (Main MCU v1.1.1)
PD3(VEL_PWR)に接続した TPS22965 ロードスイッチ(ON=アクティブHigh)で風速回路への
給電を直接 On/Off するよう変更。発熱を物理的に停止できる。

- midi_app.c: CMD_START_VEL で VEL_PWR_SetHigh(給電ON)、CMD_STOP_VEL で
  VEL_PWR_SetLow(給電OFF=発熱停止)+計測値クリア。I2C 経由の SLP/enable 制御は
  On/Off 経路から除去(PD3 が物理的に給電制御するため冗長)。velocity_enabled に
  よる計測ループの I2C ゲートは維持(給電断時の I2C ハング回避)。
- 起動時は MCC 初期値 High + velocity_enabled=true で既定 ON。
- バージョン 1.1.0 -> 1.1.1 (コマンド仕様は不変、制御方式変更を反映)。
- MCC(Melody): PD3 を GPIO 出力 VEL_PWR(初期値 High)として定義(pins.c/h, .mc3,
  manifest 更新)。
- hardware: BOM 更新。

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git_repositories\e-sensor\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6B347E-17A7-4419-94DF-B719D9ED5747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D77B6E-CC53-434E-AE4D-9BD031A3F728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41160" yWindow="1400" windowWidth="26860" windowHeight="14360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="44790" yWindow="1500" windowWidth="31010" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="e_sensor" sheetId="5" r:id="rId1"/>
@@ -479,6 +479,7 @@
   </si>
   <si>
     <t>TPS22965DSGR</t>
+    <phoneticPr fontId="19"/>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
風速計On/Offの不具合修正とバージョン更新 (Main v1.1.2 / Velocity v2 / MAUI v1.1.1)
- Velocity MCU: 5V回路On/OffをPD3(→TPS22965 ON, Active High)で制御。
  停止中はPWR_DOWNに入るとWDT(4.1s)でリセットしenable=1へ戻り5Vが
  復活する不具合を修正(常時IDLEとしwdt_resetを継続、enable=0を保持)。
- Main MCU: 風速On/OffをI2C(VELS_start/stop=enableレジスタ)で送るよう修正。
  自身のPD3を下げるだけでVelocity側へ停止が伝わらずOFFで5Vが残る不具合を解消。
- MAUI: 風速計OFF時に値を無効化(「停止中」バッジでグレー化)、ON時に予熱中
  「ウォームアップ中」バッジを表示。OffBadge文字列を追加。
- デバッグ用に15秒ごとOn/Off切替するpythonスクリプトを追加。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git_repositories\e-sensor\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D77B6E-CC53-434E-AE4D-9BD031A3F728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD72C2D7-2DC6-4F8D-8EB6-8FED5D9D12C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44790" yWindow="1500" windowWidth="31010" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="e_sensor" sheetId="5" r:id="rId1"/>

</xml_diff>